<commit_message>
Replace old data files with newly uploaded datasets
</commit_message>
<xml_diff>
--- a/Data/dim_contract.xlsx
+++ b/Data/dim_contract.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Machine Learning\Power BI\Projects\5\Dataset\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analysis\Power BI\Projects\5- Etisalat\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D355C00-FCB7-454A-90F4-C7B062FDC864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37268B51-5FC9-4451-9D2A-9AEF23038DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56350C31-280B-463A-A3AA-DD87B752F566}"/>
   </bookViews>
@@ -41,12 +41,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>Contract Key</t>
-  </si>
-  <si>
-    <t>Contract</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -63,6 +57,12 @@
   </si>
   <si>
     <t>Two Year</t>
+  </si>
+  <si>
+    <t>contract_type</t>
+  </si>
+  <si>
+    <t>contract_key</t>
   </si>
 </sst>
 </file>
@@ -446,34 +446,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>